<commit_message>
[I089] fix(checklist-requisitos): alinhar titulos repetidos com a especificacao
Acrescenta o ator, entre parenteses, ao titulo (coluna B) dos 25
requisitos cujo titulo se repetia, para coincidirem com a especificacao
de requisitos e com a RTM. Regista a alteracao na nota A2 da checklist,
que ja documenta as alteracoes anteriores (I023).

As avaliacoes dos criterios CQ-01 a CQ-11 e o resultado final de cada
requisito nao foram alterados.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04-artefactos-tecnicos/04.03-requisitos-e-rtm/m2-checklist-aprovacao-requisitos-v02.xlsx
+++ b/04-artefactos-tecnicos/04.03-requisitos-e-rtm/m2-checklist-aprovacao-requisitos-v02.xlsx
@@ -908,7 +908,7 @@
     <row r="2" ht="35.1" customHeight="1">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Katch — Grupo G11. Uma linha por requisito da Especificação de Requisitos v01 (RF001 a RF118 e RNF001 a RNF018), com o ID e o título reproduzidos do documento avaliado e uma coluna por cada critério de qualidade CQ-01 a CQ-11, pela ordem do Anexo A dos critérios. Avaliação aplicada nos termos da secção 2.1 da especificação. As linhas RF001 a RF118 mantêm a avaliação da versão v01 desta checklist; as linhas RNF001 a RNF018 foram acrescentadas pela Issue I023, depois da correção dos defeitos D01 a D08 do relatório de revisão.</t>
+          <t>Katch — Grupo G11. Uma linha por requisito da Especificação de Requisitos v01 (RF001 a RF118 e RNF001 a RNF018), com o ID e o título reproduzidos do documento avaliado e uma coluna por cada critério de qualidade CQ-01 a CQ-11, pela ordem do Anexo A dos critérios. Avaliação aplicada nos termos da secção 2.1 da especificação. As linhas RF001 a RF118 mantêm a avaliação da versão v01 desta checklist; as linhas RNF001 a RNF018 foram acrescentadas pela Issue I023, depois da correção dos defeitos D01 a D08 do relatório de revisão. Em 08-10-2026, a Issue I089 acrescentou o ator, entre parênteses, aos títulos dos 25 requisitos cujo título se repetia, para coincidirem com a Especificação de Requisitos v01 e com a RTM; as avaliações não foram alteradas.</t>
         </is>
       </c>
       <c r="B2" s="23" t="n"/>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Alterar a própria palavra-passe</t>
+          <t>Alterar a própria palavra-passe (Candidato)</t>
         </is>
       </c>
       <c r="C12" s="19" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="B37" s="19" t="inlineStr">
         <is>
-          <t>Consultar a lista de conversas</t>
+          <t>Consultar a lista de conversas (Candidato)</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="B38" s="19" t="inlineStr">
         <is>
-          <t>Consultar o histórico de uma conversa</t>
+          <t>Consultar o histórico de uma conversa (Candidato)</t>
         </is>
       </c>
       <c r="C38" s="19" t="inlineStr">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="B39" s="19" t="inlineStr">
         <is>
-          <t>Receber mensagens sem atualização manual</t>
+          <t>Receber mensagens sem atualização manual (Candidato)</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>Encerrar uma conversa</t>
+          <t>Encerrar uma conversa (Candidato)</t>
         </is>
       </c>
       <c r="C40" s="19" t="inlineStr">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="B44" s="19" t="inlineStr">
         <is>
-          <t>Consultar a área de notificações</t>
+          <t>Consultar a área de notificações (Candidato)</t>
         </is>
       </c>
       <c r="C44" s="19" t="inlineStr">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="B45" s="19" t="inlineStr">
         <is>
-          <t>Marcar notificação como lida</t>
+          <t>Marcar notificação como lida (Candidato)</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="B46" s="19" t="inlineStr">
         <is>
-          <t>Aceder ao elemento associado à notificação</t>
+          <t>Aceder ao elemento associado à notificação (Candidato)</t>
         </is>
       </c>
       <c r="C46" s="19" t="inlineStr">
@@ -3787,7 +3787,7 @@
       </c>
       <c r="B48" s="19" t="inlineStr">
         <is>
-          <t>Iniciar sessão na área de gestão web</t>
+          <t>Iniciar sessão na área de gestão web (Recrutador)</t>
         </is>
       </c>
       <c r="C48" s="19" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="B50" s="19" t="inlineStr">
         <is>
-          <t>Alterar a própria palavra-passe</t>
+          <t>Alterar a própria palavra-passe (Recrutador)</t>
         </is>
       </c>
       <c r="C50" s="19" t="inlineStr">
@@ -6163,7 +6163,7 @@
       </c>
       <c r="B81" s="19" t="inlineStr">
         <is>
-          <t>Consultar a lista de conversas</t>
+          <t>Consultar a lista de conversas (Recrutador)</t>
         </is>
       </c>
       <c r="C81" s="19" t="inlineStr">
@@ -6235,7 +6235,7 @@
       </c>
       <c r="B82" s="19" t="inlineStr">
         <is>
-          <t>Consultar o histórico de uma conversa</t>
+          <t>Consultar o histórico de uma conversa (Recrutador)</t>
         </is>
       </c>
       <c r="C82" s="19" t="inlineStr">
@@ -6307,7 +6307,7 @@
       </c>
       <c r="B83" s="19" t="inlineStr">
         <is>
-          <t>Receber mensagens sem atualização manual</t>
+          <t>Receber mensagens sem atualização manual (Recrutador)</t>
         </is>
       </c>
       <c r="C83" s="19" t="inlineStr">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="B84" s="19" t="inlineStr">
         <is>
-          <t>Encerrar uma conversa</t>
+          <t>Encerrar uma conversa (Recrutador)</t>
         </is>
       </c>
       <c r="C84" s="19" t="inlineStr">
@@ -6811,7 +6811,7 @@
       </c>
       <c r="B90" s="19" t="inlineStr">
         <is>
-          <t>Consultar a área de notificações</t>
+          <t>Consultar a área de notificações (Recrutador)</t>
         </is>
       </c>
       <c r="C90" s="19" t="inlineStr">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="B91" s="19" t="inlineStr">
         <is>
-          <t>Marcar notificação como lida</t>
+          <t>Marcar notificação como lida (Recrutador)</t>
         </is>
       </c>
       <c r="C91" s="19" t="inlineStr">
@@ -6955,7 +6955,7 @@
       </c>
       <c r="B92" s="19" t="inlineStr">
         <is>
-          <t>Aceder ao elemento associado à notificação</t>
+          <t>Aceder ao elemento associado à notificação (Recrutador)</t>
         </is>
       </c>
       <c r="C92" s="19" t="inlineStr">
@@ -7027,7 +7027,7 @@
       </c>
       <c r="B93" s="19" t="inlineStr">
         <is>
-          <t>Iniciar sessão na área de gestão web</t>
+          <t>Iniciar sessão na área de gestão web (Administrador)</t>
         </is>
       </c>
       <c r="C93" s="19" t="inlineStr">
@@ -7099,7 +7099,7 @@
       </c>
       <c r="B94" s="19" t="inlineStr">
         <is>
-          <t>Alterar a própria palavra-passe</t>
+          <t>Alterar a própria palavra-passe (Administrador)</t>
         </is>
       </c>
       <c r="C94" s="19" t="inlineStr">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="B116" s="19" t="inlineStr">
         <is>
-          <t>Terminar sessão na área de gestão web</t>
+          <t>Terminar sessão na área de gestão web (Recrutador)</t>
         </is>
       </c>
       <c r="C116" s="19" t="inlineStr">
@@ -8755,7 +8755,7 @@
       </c>
       <c r="B117" s="19" t="inlineStr">
         <is>
-          <t>Terminar sessão na área de gestão web</t>
+          <t>Terminar sessão na área de gestão web (Administrador)</t>
         </is>
       </c>
       <c r="C117" s="19" t="inlineStr">
@@ -8827,7 +8827,7 @@
       </c>
       <c r="B118" s="19" t="inlineStr">
         <is>
-          <t>Marcar como lidas as mensagens ao abrir a conversa</t>
+          <t>Marcar como lidas as mensagens ao abrir a conversa (Candidato)</t>
         </is>
       </c>
       <c r="C118" s="19" t="inlineStr">
@@ -8899,7 +8899,7 @@
       </c>
       <c r="B119" s="19" t="inlineStr">
         <is>
-          <t>Marcar como lidas as mensagens ao abrir a conversa</t>
+          <t>Marcar como lidas as mensagens ao abrir a conversa (Recrutador)</t>
         </is>
       </c>
       <c r="C119" s="19" t="inlineStr">
@@ -8971,7 +8971,7 @@
       </c>
       <c r="B120" s="19" t="inlineStr">
         <is>
-          <t>Receber notificações sem atualização manual</t>
+          <t>Receber notificações sem atualização manual (Candidato)</t>
         </is>
       </c>
       <c r="C120" s="19" t="inlineStr">
@@ -9043,7 +9043,7 @@
       </c>
       <c r="B121" s="19" t="inlineStr">
         <is>
-          <t>Receber notificações sem atualização manual</t>
+          <t>Receber notificações sem atualização manual (Recrutador)</t>
         </is>
       </c>
       <c r="C121" s="19" t="inlineStr">

</xml_diff>